<commit_message>
data: real transfer pricing for Cervinia, Grandvalira, Pamporovo
All three had ZERO curated transfer rows -- silently falling back to
the legacy distance-based formula that transfers.py's own module
docstring already calls "a fudge matching no real pricing structure".
These three are the same skideal.co.il-confirmed resorts as the
terrain-data commit just before this one.

- Cervinia (via MXP), Grandvalira (via BCN): real current pricing
  found and sourced (shared shuttle + private transfer each).
- Pamporovo (via PDV): best source found was an explicitly archived
  2022-23 winter rate card -- no current-season pricing turned up
  despite a real search effort. Added as 'estimated', not 'sourced',
  rather than passing a 3-year-old number off as current.
</commit_message>
<xml_diff>
--- a/data/transfer_options.xlsx
+++ b/data/transfer_options.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TransferOptions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Method" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="TransferOptions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Notes &amp; Method" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M60"/>
+  <dimension ref="A1:M66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3958,6 +3958,363 @@
       <c r="M60" s="5" t="inlineStr">
         <is>
           <t>Comparable to the Geneva private rate for a similar distance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>MXP</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Cervinia (Breuil-Cervinia)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>shared_shuttle</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>70</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>per_person</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>165</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>SkiHolidayTransfers / Alps2Alps</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>EUR70pp winter season via skiholidaytransfers.com; Alps2Alps quotes 'from EUR50pp' as a lower headline figure. 2-3h10 journey depending on source; 165min used to match this resort's existing transfer_minutes_by_airport.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>MXP</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Cervinia (Breuil-Cervinia)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>private_transfer</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>516</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>per_vehicle</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>8</v>
+      </c>
+      <c r="G62" t="n">
+        <v>165</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>SkiHolidayTransfers</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>EUR516 total via skiholidaytransfers.com ('starting from'); vehicle capacity not stated on the source page -- 8 assumed, matching this dataset's standard private-minivan convention elsewhere (e.g. Chamonix, Grandvalira), not a source-confirmed number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>BCN</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Grandvalira (Andorra)</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>shared_shuttle</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>72</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>per_person</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>190</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Alps2Alps / various</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>EUR72pp 'starting from', Barcelona to Pas de la Casa (a Grandvalira sector), ~3h10 journey.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>BCN</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Grandvalira (Andorra)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>private_transfer</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>240</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>per_vehicle</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>8</v>
+      </c>
+      <c r="G64" t="n">
+        <v>180</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Chofix</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>EUR240 for an Opel Vivaro (up to 8 passengers) via chofix.com's published vehicle-tier pricing; taxes/tips included per that page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>PDV</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Pamporovo</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>shared_shuttle</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>35</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>per_person</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>90</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Pamporovo Express</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>estimated</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>2-person tier from an ARCHIVED 2022-23 winter rate card (pamporovoexpress.com/prices, page itself flags these dates) -- no current-season source found despite a real search effort. Directionally real, not verified current.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>PDV</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Pamporovo</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>private_transfer</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>119</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>per_vehicle</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>8</v>
+      </c>
+      <c r="G66" t="n">
+        <v>90</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Pamporovo Express</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>estimated</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>5-8 person tier from the same archived 2022-23 rate card as the shared_shuttle row above -- same staleness caveat.</t>
         </is>
       </c>
     </row>

</xml_diff>